<commit_message>
fixed resolution count visual bug
</commit_message>
<xml_diff>
--- a/docs/data/sample4.xlsx
+++ b/docs/data/sample4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\erenimo\projects\ses\docs\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0904723E-8E40-4898-B982-2F952EBACE59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB821CAC-6561-4724-9325-847C12E86848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1815" yWindow="1815" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2850" yWindow="2850" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Page 1" sheetId="1" r:id="rId1"/>
@@ -38,9 +38,6 @@
     <t>No_0833AB</t>
   </si>
   <si>
-    <t>Öğrenci No_0833AB</t>
-  </si>
-  <si>
     <t>Adı_0833AB</t>
   </si>
   <si>
@@ -65,12 +62,6 @@
     <t>2</t>
   </si>
   <si>
-    <t>Midterm(%25)_0833AB</t>
-  </si>
-  <si>
-    <t>Attendance(%25)_0833AB</t>
-  </si>
-  <si>
     <t>Final(%40)_0833AB</t>
   </si>
   <si>
@@ -93,6 +84,15 @@
   </si>
   <si>
     <t>221400025</t>
+  </si>
+  <si>
+    <t>Öğrenci No_0833AB</t>
+  </si>
+  <si>
+    <t>Midterm(%25)_0833AB</t>
+  </si>
+  <si>
+    <t>Attendance(%25)_0833AB</t>
   </si>
 </sst>
 </file>
@@ -1411,101 +1411,101 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>8</v>
-      </c>
       <c r="F2" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G2" s="9">
         <v>80</v>
       </c>
       <c r="H2" s="9">
         <f ca="1">TRUNC(60 + ((RAND()*100 - 0) * (100 - 60) / (100 - 0)))</f>
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="I2" s="9">
         <f ca="1">TRUNC(30 + ((RAND()*100 - 0) * (60 - 30) / (100 - 0)))</f>
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="J2" s="9">
         <f ca="1">TRUNC(30 + ((RAND()*100 - 0) * (60 - 30) / (100 - 0)))</f>
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="K2" s="6"/>
     </row>
     <row r="3" spans="1:11" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G3" s="9">
         <v>125</v>
       </c>
       <c r="H3" s="9">
-        <f t="shared" ref="G3:H25" ca="1" si="0">TRUNC(60 + ((RAND()*100 - 0) * (100 - 60) / (100 - 0)))</f>
-        <v>95</v>
+        <f t="shared" ref="H3" ca="1" si="0">TRUNC(60 + ((RAND()*100 - 0) * (100 - 60) / (100 - 0)))</f>
+        <v>94</v>
       </c>
       <c r="I3" s="9">
-        <f t="shared" ref="I3:J25" ca="1" si="1">TRUNC(30 + ((RAND()*100 - 0) * (60 - 30) / (100 - 0)))</f>
-        <v>31</v>
+        <f t="shared" ref="I3" ca="1" si="1">TRUNC(30 + ((RAND()*100 - 0) * (60 - 30) / (100 - 0)))</f>
+        <v>54</v>
       </c>
       <c r="J3" s="9">
         <v>80</v>

</xml_diff>